<commit_message>
Refresh FRS assets and fixtures for EJAM 3.2022.3
</commit_message>
<xml_diff>
--- a/inst/testdata/programid/testinput_program_sys_id_8.xlsx
+++ b/inst/testdata/programid/testinput_program_sys_id_8.xlsx
@@ -20,52 +20,52 @@
     <t xml:space="preserve">PRIMARY_NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">FIS:7-0540-00003, NPDES:NY0153745</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEJAMADA CAMPGROUND &amp; RV PARK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:354362</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KREJAM CORP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMS:1513529</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEJAME &amp; SONS INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:485659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA VEJAMA DISCOUNT STORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NPDES:LAG750956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRACEJAMES ENT, LLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RCRAINFO:CAC002995519</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEJAMIN HAFERTEPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601252181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601439158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC</t>
+    <t xml:space="preserve">NPDES:01R10I002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DYNAMITE PICKLEBALL OF MERRIMACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCRAINFO:AK0000000323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA USFS R10 CHUGACH NF CORDOVA FOREST WORK C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EIS:14548611, TRIS:0000WFWRRN9CESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.E. WARREN AIR FORCE BASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:0100000009003E0010, CEDRI:CEDRI101781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIGHLAND PARK MARKET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SFDW:020000015, SFDW:020000015 0000015TP004, SFDW:NY3120465, SFDW:NY3120465 15711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TUSCARORA NATION SCHOOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGRID:57187, EIA-860:57187, SEMS:AK0000042325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PILLAR MOUNTAIN WIND PROJECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:WANCA0005307300037, AIRS/AFS:5307300037, CAMDBS:54537, E-GGRT:1000001, EGRID:54537, EIA-860:54537, EIS:6212611, ICIS:3000006257, NPDES:WA0031291, RCRAINFO:WAR000007823, RCRAINFO:WAY000203463, TRIS:98248TNSKW5105L, WA-FSIS:92884494</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TENASKA COGENERATION PLANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR:AK0000882274, CEDRI:CEDRI10258451</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTCO WHOLESALE #63</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Refresh FRS datasets and fixtures for EJAM 3.2022.3 (#626)
* Refresh FRS assets and fixtures for EJAM 3.2022.3

* Restamp compatible ejamdata Arrow asset metadata

* Normalize MACT labels for FRS refresh

* fixed glitch in document() re imports like graphics vs terra

* documentation of frs changes

* ejamdata_version updated to v3.2022.3

this makes it use the updated frs datasets that are assets in the ejamdata repository

* remove library(arrow) and desc from a script just to quiet any flags in checks

* Mock GitHub token selection in release asset test

* minor fixes to check() warnings
</commit_message>
<xml_diff>
--- a/inst/testdata/programid/testinput_program_sys_id_8.xlsx
+++ b/inst/testdata/programid/testinput_program_sys_id_8.xlsx
@@ -20,52 +20,52 @@
     <t xml:space="preserve">PRIMARY_NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">FIS:7-0540-00003, NPDES:NY0153745</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEJAMADA CAMPGROUND &amp; RV PARK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:354362</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KREJAM CORP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMS:1513529</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEJAME &amp; SONS INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:485659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA VEJAMA DISCOUNT STORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NPDES:LAG750956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRACEJAMES ENT, LLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RCRAINFO:CAC002995519</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEJAMIN HAFERTEPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601252181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601439158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC</t>
+    <t xml:space="preserve">NPDES:01R10I002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DYNAMITE PICKLEBALL OF MERRIMACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCRAINFO:AK0000000323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA USFS R10 CHUGACH NF CORDOVA FOREST WORK C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EIS:14548611, TRIS:0000WFWRRN9CESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.E. WARREN AIR FORCE BASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:0100000009003E0010, CEDRI:CEDRI101781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIGHLAND PARK MARKET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SFDW:020000015, SFDW:020000015 0000015TP004, SFDW:NY3120465, SFDW:NY3120465 15711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TUSCARORA NATION SCHOOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGRID:57187, EIA-860:57187, SEMS:AK0000042325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PILLAR MOUNTAIN WIND PROJECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:WANCA0005307300037, AIRS/AFS:5307300037, CAMDBS:54537, E-GGRT:1000001, EGRID:54537, EIA-860:54537, EIS:6212611, ICIS:3000006257, NPDES:WA0031291, RCRAINFO:WAR000007823, RCRAINFO:WAY000203463, TRIS:98248TNSKW5105L, WA-FSIS:92884494</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TENASKA COGENERATION PLANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR:AK0000882274, CEDRI:CEDRI10258451</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTCO WHOLESALE #63</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
v3.2022.3 version bump to prep release of last version using frozen ACS 2018-2022 vintage datasets (#627)
* ejamdata_required_tag: v3.2022.3

Will require a new set of files as assets in ejamdata repo

* Refresh FRS datasets and fixtures for EJAM 3.2022.3 (#626)

* Refresh FRS assets and fixtures for EJAM 3.2022.3

* Restamp compatible ejamdata Arrow asset metadata

* Normalize MACT labels for FRS refresh

* fixed glitch in document() re imports like graphics vs terra

* documentation of frs changes

* ejamdata_version updated to v3.2022.3

this makes it use the updated frs datasets that are assets in the ejamdata repository

* remove library(arrow) and desc from a script just to quiet any flags in checks

* Mock GitHub token selection in release asset test

* minor fixes to check() warnings

* Register MACT label test in FRS test group

* Recognize release documentation terms in spelling check
</commit_message>
<xml_diff>
--- a/inst/testdata/programid/testinput_program_sys_id_8.xlsx
+++ b/inst/testdata/programid/testinput_program_sys_id_8.xlsx
@@ -20,52 +20,52 @@
     <t xml:space="preserve">PRIMARY_NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">FIS:7-0540-00003, NPDES:NY0153745</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEJAMADA CAMPGROUND &amp; RV PARK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:354362</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KREJAM CORP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMS:1513529</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEJAME &amp; SONS INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NJ-NJEMS:485659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA VEJAMA DISCOUNT STORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NPDES:LAG750956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRACEJAMES ENT, LLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RCRAINFO:CAC002995519</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEJAMIN HAFERTEPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601252181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIS:3601439158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJAM INC</t>
+    <t xml:space="preserve">NPDES:01R10I002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DYNAMITE PICKLEBALL OF MERRIMACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCRAINFO:AK0000000323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA USFS R10 CHUGACH NF CORDOVA FOREST WORK C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EIS:14548611, TRIS:0000WFWRRN9CESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.E. WARREN AIR FORCE BASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:0100000009003E0010, CEDRI:CEDRI101781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIGHLAND PARK MARKET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SFDW:020000015, SFDW:020000015 0000015TP004, SFDW:NY3120465, SFDW:NY3120465 15711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TUSCARORA NATION SCHOOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGRID:57187, EIA-860:57187, SEMS:AK0000042325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PILLAR MOUNTAIN WIND PROJECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR:WANCA0005307300037, AIRS/AFS:5307300037, CAMDBS:54537, E-GGRT:1000001, EGRID:54537, EIA-860:54537, EIS:6212611, ICIS:3000006257, NPDES:WA0031291, RCRAINFO:WAR000007823, RCRAINFO:WAY000203463, TRIS:98248TNSKW5105L, WA-FSIS:92884494</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TENASKA COGENERATION PLANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR:AK0000882274, CEDRI:CEDRI10258451</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTCO WHOLESALE #63</t>
   </si>
 </sst>
 </file>

</xml_diff>